<commit_message>
Correct 2026 teaching program release basis
</commit_message>
<xml_diff>
--- a/assets/teacher/delivery-register-v1.0.0.xlsx
+++ b/assets/teacher/delivery-register-v1.0.0.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Register" sheetId="1" r:id="Reac353b174504be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher confirmations" sheetId="2" r:id="Rf83b9857dd334bf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source and links" sheetId="3" r:id="R3684c10a4ad54ba1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Register" sheetId="1" r:id="Ra1f256c73d8a439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher confirmations" sheetId="2" r:id="Rcf6fec1fabe748ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source and links" sheetId="3" r:id="R0bd3b549e231403c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2024,7 +2024,7 @@
         <x:v>TC-01</x:v>
       </x:c>
       <x:c r="B5" s="34" t="str">
-        <x:v>Delivery year, timetable pattern and total course hours</x:v>
+        <x:v>Timetable pattern and total course hours</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
         <x:v>Controls usable pacing and reporting claims.</x:v>
@@ -2036,7 +2036,7 @@
         <x:v>Before program approval</x:v>
       </x:c>
       <x:c r="F5" s="34" t="str">
-        <x:v>Enter the confirmed year, periods per cycle and total hours.</x:v>
+        <x:v>Enter the confirmed periods per cycle and total hours.</x:v>
       </x:c>
       <x:c r="G5" s="43" t="str">
         <x:v>Teacher to confirm</x:v>
@@ -2255,7 +2255,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="21.600000381469727" hidden="0" customHeight="1">
+    <x:row r="5" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A5" s="34" t="str">
         <x:v>Official NESA Graphics Technology 7–10 syllabus page</x:v>
       </x:c>
@@ -2263,7 +2263,7 @@
         <x:v>Official curriculum</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>Current/default syllabus pathway for 2026–2027.</x:v>
+        <x:v>Selected Graphics Technology 2019 / GT5 pathway for the confirmed 2026 course.</x:v>
       </x:c>
       <x:c r="D5" s="46" t="str">
         <x:v>https://www.nsw.gov.au/education-and-training/nesa/curriculum/tas/graphics-technology-7-10-2019</x:v>
@@ -2272,7 +2272,7 @@
         <x:v>30/08/2026</x:v>
       </x:c>
       <x:c r="F5" s="34" t="str">
-        <x:v>New Communication Technology syllabus begins in 2028; do not mix the two pathways.</x:v>
+        <x:v>Communication Technology 2025 may be adopted early by schools in 2026–2027 and is mandatory from 2028; Graphics Technology 2019 remains available through December 2029. Do not mix pathways.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">

</xml_diff>